<commit_message>
Registro de cambios de recepciones (quién, qué y cuándo)
- Migraciones 008-009: tabla audit_log y triggers que anotan la creación,
  modificación (campos, palets, defectos, fotos) y eliminación de recepciones;
  solo lectura para el administrador
- Maestros -> Registro: listado con búsqueda y filtro por acción, con los
  cambios descritos en lenguaje claro (antes -> después)
- Los guardados sin cambios reales no aparecen

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/USUARIOS.xlsx
+++ b/USUARIOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://frunetbio.sharepoint.com/sites/FRUNET/Documentos compartidos/ADMON Y FINANZAS/CONTROL/PROYECTOS APP/APP CALIDAD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D87C9058-2E52-4A2E-9C9F-6D56125B6CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{D87C9058-2E52-4A2E-9C9F-6D56125B6CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B75C68AA-09C0-434B-BFC9-E07FFDC89189}"/>
   <bookViews>
     <workbookView xWindow="255" yWindow="0" windowWidth="28545" windowHeight="15600" xr2:uid="{5EB75800-834E-41FB-8CE0-5FC8B498DEAC}"/>
   </bookViews>
@@ -433,6 +433,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D158D488-A181-4B1D-BBBD-D1F9E17A2A66}">
   <dimension ref="C7:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="7" spans="3:5" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
@@ -493,6 +497,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1999b526-aaa7-4ee2-8538-819e083ff1a3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="4fdfdd06-c627-4a34-bd2a-a802ea236432" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101009DD8FCA63F874348AB49A0F66113FAF6" ma:contentTypeVersion="19" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="b34882c4ae77072a31d932a494fc8eed">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4fdfdd06-c627-4a34-bd2a-a802ea236432" xmlns:ns3="1999b526-aaa7-4ee2-8538-819e083ff1a3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f5f6a96ed0619fe0835755c5186181c" ns2:_="" ns3:_="">
     <xsd:import namespace="4fdfdd06-c627-4a34-bd2a-a802ea236432"/>
@@ -753,34 +777,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1999b526-aaa7-4ee2-8538-819e083ff1a3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="4fdfdd06-c627-4a34-bd2a-a802ea236432" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5B32DC9-8A14-4CC6-AF23-910EBC44527E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7E47F96-12D7-49CF-BF12-77CA2CA43822}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="1999b526-aaa7-4ee2-8538-819e083ff1a3"/>
+    <ds:schemaRef ds:uri="4fdfdd06-c627-4a34-bd2a-a802ea236432"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FD6D1B7-F230-439C-B94B-40650DA9D70C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7FD6D1B7-F230-439C-B94B-40650DA9D70C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7E47F96-12D7-49CF-BF12-77CA2CA43822}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5B32DC9-8A14-4CC6-AF23-910EBC44527E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4fdfdd06-c627-4a34-bd2a-a802ea236432"/>
+    <ds:schemaRef ds:uri="1999b526-aaa7-4ee2-8538-819e083ff1a3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>